<commit_message>
fidelity 401k netbenefits from CSV only; bofa description fix
</commit_message>
<xml_diff>
--- a/tests/fixtures/vanguard-brokerage-xlsx-synthetic-sample.xlsx
+++ b/tests/fixtures/vanguard-brokerage-xlsx-synthetic-sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Transaction History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaction History" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -845,33 +845,113 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DISCLOSURES</t>
-        </is>
-      </c>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>VFIAX</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Vanguard 500 Index Fund Admiral</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>100.0000</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>*Note on account protection: Securities in your brokerage account are held in custody by a synthetic custodian for this test fixture.</t>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>VMFXX</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Vanguard Federal Money Market Fund</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sweep in</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-$25.00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>**The fees displayed include but are not limited to commissions and transaction fees. This is invented text for a test fixture.</t>
+          <t>DISCLOSURES</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>This report is not intended to replace an account statement or confirmation.</t>
+          <t>*Note on account protection: Securities in your brokerage account are held in custody by a synthetic custodian for this test fixture.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>**The fees displayed include but are not limited to commissions and transaction fees. This is invented text for a test fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>This report is not intended to replace an account statement or confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>(C) 2026 Synthetic Test Data. Not a real Vanguard document.</t>
         </is>

</xml_diff>

<commit_message>
fidelity 401k netbenefits from CSV only; bofa description fix (#8)
</commit_message>
<xml_diff>
--- a/tests/fixtures/vanguard-brokerage-xlsx-synthetic-sample.xlsx
+++ b/tests/fixtures/vanguard-brokerage-xlsx-synthetic-sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Transaction History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaction History" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -845,33 +845,113 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DISCLOSURES</t>
-        </is>
-      </c>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>VFIAX</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Vanguard 500 Index Fund Admiral</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Transfer</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>100.0000</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>*Note on account protection: Securities in your brokerage account are held in custody by a synthetic custodian for this test fixture.</t>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4/09/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>VMFXX</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Vanguard Federal Money Market Fund</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sweep in</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-$25.00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>**The fees displayed include but are not limited to commissions and transaction fees. This is invented text for a test fixture.</t>
+          <t>DISCLOSURES</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>This report is not intended to replace an account statement or confirmation.</t>
+          <t>*Note on account protection: Securities in your brokerage account are held in custody by a synthetic custodian for this test fixture.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>**The fees displayed include but are not limited to commissions and transaction fees. This is invented text for a test fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>This report is not intended to replace an account statement or confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>(C) 2026 Synthetic Test Data. Not a real Vanguard document.</t>
         </is>

</xml_diff>